<commit_message>
I filled out an additional part of the conducted tests.
</commit_message>
<xml_diff>
--- a/6_QA/Тестирование Наш Слон.xlsx
+++ b/6_QA/Тестирование Наш Слон.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Владимир\AIMessenger\6_QA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28EF2A23-701D-45E0-BA1B-2F435C2D841F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD55FB34-61A9-469A-AB6C-61045DBD90BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="21429" activeTab="2" xr2:uid="{100470D7-4961-4BE2-8F1F-B36A2B568951}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="21429" activeTab="1" xr2:uid="{100470D7-4961-4BE2-8F1F-B36A2B568951}"/>
   </bookViews>
   <sheets>
     <sheet name="Авторизация и регистрация" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="445" uniqueCount="201">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="514" uniqueCount="230">
   <si>
     <t>Номер п/п</t>
   </si>
@@ -666,6 +666,99 @@
   </si>
   <si>
     <t>После полного выхода и закрытия мессенджера, а затем последующего входа в мессенджер в свой аккаунт и переход на вкладку "Контакты", корректно отображает сформированный ранее текущим пользователем "Список сотрудников и участников" при входе в свой аккаунт с разных устройств.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Нажать на кнопку "Новый чат" в левом верхнем углу, находясь на любой странице мессенджера, выбрать в поле ниже "Контакты" "Список сотрудников и участников" одного из контрагентов, представленных в списке. В открывшейся "Карточке контакта" нажать "Написать" в правом верхнем углу текущей страницы. </t>
+  </si>
+  <si>
+    <t>Открывается окно чата с выбранным контактом.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Нажать на вкладку/кнопку "Личные сообщения" в левом верхнем углу, находясь на любой странице мессенджера, выбрать чат с одним из контрагентов в открывшемся в списке "Личные сообщения" "Личные диалоги с участниками команды". </t>
+  </si>
+  <si>
+    <t>Возможность удаления выбранного чата / чатов из списка "Личные сообщения" "Личные диалоги с участниками команды".</t>
+  </si>
+  <si>
+    <t>Не пройдено</t>
+  </si>
+  <si>
+    <t>Критическая</t>
+  </si>
+  <si>
+    <t>Не обнаружена кнопка "Удалить", возможность удалить отсутствует и при открытии меню правой кнопки мыши, как при выборе чата, так и при нажатии на него. Отсутствует возможность удалить сообщения внутри чата.</t>
+  </si>
+  <si>
+    <t>Создание и отправка сообщения в личном чате.</t>
+  </si>
+  <si>
+    <t>Страница "Личные сообщения" "Личные диалоги с участниками команды" мессенджера.</t>
+  </si>
+  <si>
+    <t>Сообщение создается и отправляется.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">В открывшемся окне нового или уже существующего чата в поле внизу страницы обычное текстовое сообщение вводится и отправляется.  
+В сообщение можно добавить смайлики, при этом отправка и получение сообщения происходит корректно.
+При попытке добавить в сообщение вложенный файл размером около 5Mb и отправке его произошло зависание мессенджера, в том числе, и у других пользователей. Сообщение отправлено не было.  </t>
+  </si>
+  <si>
+    <t>Создание нового группового чата с одним участником.</t>
+  </si>
+  <si>
+    <t>Создание нового группового чата с двумя и более участниками.</t>
+  </si>
+  <si>
+    <t>Нажать на кнопку "Новый чат" или "Личные сообщения" в левом верхнем углу, находясь на любой странице мессенджера, выбрать чат с одним из контрагентов в открывшемся в списке "Личные сообщения" "Личные диалоги с участниками команды". В открывшемся окне чата внизу страницы ввести сообщение для выбранного контакта и отправить его.</t>
+  </si>
+  <si>
+    <t>Создание нового группового чата</t>
+  </si>
+  <si>
+    <t>Нажать на вкладку/кнопку "Корпоративные чаты" в левой части страницы, на загрузившейся странице нажать на кнопку "Создать группу" в правом верхнем углу. В открывшемся окне "Создание группы" заполнить поля "Название группы" "Описание", поставить галочки на выбранных участниках из ранее сформированного списка контрагентов. Нажать кнопку "Создать группу" в нижней части модуля "Создание группы".</t>
+  </si>
+  <si>
+    <t>Нажать на вкладку/кнопку "Корпоративные чаты" в левой части страницы, на загрузившейся странице нажать на кнопку "Создать группу" в правом верхнем углу. В открывшемся окне "Создание группы" заполнить поля "Название группы" "Описание", поставить галочку на одном из контактов из ранее сформированного списка контрагентов. Нажать кнопку "Создать группу" в нижней части модуля "Создание группы".</t>
+  </si>
+  <si>
+    <t>Создание нового группового чата с несколькими участниками</t>
+  </si>
+  <si>
+    <t>Выполнение всех шагов проверки корректно создает новый групповой чат и добавляет в него выбранных участников из списка контактов текущего пользователя.</t>
+  </si>
+  <si>
+    <t>Выполнение всех шагов проверки корректно создает новый групповой чат и добавляет в него выбранного участника из списка контактов текущего пользователя.</t>
+  </si>
+  <si>
+    <t>Страница "Групповые чаты" мессенджера.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Открытая вкладка мессенджера "Корпоративные чаты" </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Нажать на вкладку/кнопку "Удалить" или выбрать соответствующую команду из контектстного меню, открывающегося при нажатии правой кнопки мыши </t>
+  </si>
+  <si>
+    <t>Возможность удаления выбранного одного или более участников из группового чата.</t>
+  </si>
+  <si>
+    <t>Не обнаружена кнопка/вкладка "Удалить", возможность удалить отсутствует и при открытии меню правой кнопки мыши, как при выборе чата, так и при нажатии на него. Отсутствует возможность удалить участников внутри чата.</t>
+  </si>
+  <si>
+    <t>Не обнаружена кнопка/вкладка "Удалить", возможность удалить отсутствует и при открытии меню правой кнопки мыши, как при выборе чата, так и при нажатии на него. Отсутствует возможность удалить выбранный чат внутри него самого.</t>
+  </si>
+  <si>
+    <t>Создание и отправка сообщения в групповом чате.</t>
+  </si>
+  <si>
+    <t>Нажать на выбранный чат в открывшемся в списке "Групповые чаты". В открывшемся окне чата внизу страницы ввести сообщение для всех участников чата и отправить его.</t>
+  </si>
+  <si>
+    <t>В открывшемся окне существующего чата в поле внизу страницы обычное текстовое сообщение вводится и отправляется.  
+В сообщение можно добавить смайлики, при этом отправка и получение сообщения происходит корректно.
+При попытке добавить в сообщение вложенный файл размером около 1Mb и отправке его произошло зависание мессенджера, в том числе, и у других пользователей. 
+Сообщение отправлено не было и потом исчезло. 
+Мессенджер при этом остался в работоспособном состоянии.</t>
   </si>
 </sst>
 </file>
@@ -892,7 +985,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -918,9 +1011,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -945,6 +1035,18 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1276,38 +1378,38 @@
     <col min="11" max="11" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="9" t="s">
+    <row r="1" spans="1:16" s="21" customFormat="1" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="D1" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="E1" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="F1" s="10" t="s">
+      <c r="F1" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="G1" s="10" t="s">
+      <c r="G1" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="H1" s="10" t="s">
+      <c r="H1" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="I1" s="10" t="s">
+      <c r="I1" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="J1" s="10" t="s">
+      <c r="J1" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="K1" s="11" t="s">
+      <c r="K1" s="20" t="s">
         <v>24</v>
       </c>
     </row>
@@ -1345,7 +1447,7 @@
       </c>
     </row>
     <row r="3" spans="1:16" s="1" customFormat="1" ht="72.900000000000006" hidden="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="15"/>
+      <c r="A3" s="12"/>
       <c r="B3" s="3" t="s">
         <v>3</v>
       </c>
@@ -1367,10 +1469,10 @@
       <c r="J3" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="K3" s="16"/>
+      <c r="K3" s="13"/>
     </row>
     <row r="4" spans="1:16" ht="29.15" x14ac:dyDescent="0.4">
-      <c r="A4" s="17">
+      <c r="A4" s="14">
         <v>1</v>
       </c>
       <c r="B4" s="2" t="s">
@@ -1389,7 +1491,7 @@
       <c r="G4" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="H4" s="20" t="s">
+      <c r="H4" s="17" t="s">
         <v>46</v>
       </c>
       <c r="I4" s="2" t="s">
@@ -1406,7 +1508,7 @@
       <c r="P4" s="1"/>
     </row>
     <row r="5" spans="1:16" ht="43.75" x14ac:dyDescent="0.4">
-      <c r="A5" s="17">
+      <c r="A5" s="14">
         <f>A4+1</f>
         <v>2</v>
       </c>
@@ -1428,7 +1530,7 @@
       <c r="G5" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="H5" s="20" t="s">
+      <c r="H5" s="17" t="s">
         <v>46</v>
       </c>
       <c r="I5" s="2" t="s">
@@ -1437,7 +1539,7 @@
       <c r="J5" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="K5" s="18"/>
+      <c r="K5" s="15"/>
       <c r="L5" s="1"/>
       <c r="M5" s="1"/>
       <c r="N5" s="1"/>
@@ -1445,7 +1547,7 @@
       <c r="P5" s="1"/>
     </row>
     <row r="6" spans="1:16" ht="58.3" x14ac:dyDescent="0.4">
-      <c r="A6" s="17">
+      <c r="A6" s="14">
         <f t="shared" ref="A6:A37" si="0">A5+1</f>
         <v>3</v>
       </c>
@@ -1467,7 +1569,7 @@
       <c r="G6" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="H6" s="20" t="s">
+      <c r="H6" s="17" t="s">
         <v>46</v>
       </c>
       <c r="I6" s="2" t="s">
@@ -1484,7 +1586,7 @@
       <c r="P6" s="1"/>
     </row>
     <row r="7" spans="1:16" ht="42.9" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="17">
+      <c r="A7" s="14">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
@@ -1506,7 +1608,7 @@
       <c r="G7" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="H7" s="20" t="s">
+      <c r="H7" s="17" t="s">
         <v>46</v>
       </c>
       <c r="I7" s="2" t="s">
@@ -1518,7 +1620,7 @@
       <c r="K7" s="2"/>
     </row>
     <row r="8" spans="1:16" ht="181.3" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A8" s="17">
+      <c r="A8" s="14">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
@@ -1540,7 +1642,7 @@
       <c r="G8" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="H8" s="20" t="s">
+      <c r="H8" s="17" t="s">
         <v>46</v>
       </c>
       <c r="I8" s="2" t="s">
@@ -1554,7 +1656,7 @@
       </c>
     </row>
     <row r="9" spans="1:16" ht="63.45" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A9" s="17">
+      <c r="A9" s="14">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
@@ -1576,7 +1678,7 @@
       <c r="G9" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="H9" s="20" t="s">
+      <c r="H9" s="17" t="s">
         <v>46</v>
       </c>
       <c r="I9" s="2" t="s">
@@ -1588,7 +1690,7 @@
       <c r="K9" s="2"/>
     </row>
     <row r="10" spans="1:16" ht="87.45" x14ac:dyDescent="0.4">
-      <c r="A10" s="17">
+      <c r="A10" s="14">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
@@ -1610,7 +1712,7 @@
       <c r="G10" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="H10" s="20" t="s">
+      <c r="H10" s="17" t="s">
         <v>65</v>
       </c>
       <c r="I10" s="2" t="s">
@@ -1624,7 +1726,7 @@
       </c>
     </row>
     <row r="11" spans="1:16" ht="87.45" x14ac:dyDescent="0.4">
-      <c r="A11" s="17">
+      <c r="A11" s="14">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
@@ -1646,7 +1748,7 @@
       <c r="G11" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="H11" s="20" t="s">
+      <c r="H11" s="17" t="s">
         <v>46</v>
       </c>
       <c r="I11" s="2" t="s">
@@ -1658,7 +1760,7 @@
       <c r="K11" s="2"/>
     </row>
     <row r="12" spans="1:16" ht="87.45" x14ac:dyDescent="0.4">
-      <c r="A12" s="17">
+      <c r="A12" s="14">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
@@ -1680,7 +1782,7 @@
       <c r="G12" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="H12" s="20" t="s">
+      <c r="H12" s="17" t="s">
         <v>46</v>
       </c>
       <c r="I12" s="2" t="s">
@@ -1692,7 +1794,7 @@
       <c r="K12" s="2"/>
     </row>
     <row r="13" spans="1:16" ht="102" x14ac:dyDescent="0.4">
-      <c r="A13" s="17">
+      <c r="A13" s="14">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
@@ -1714,7 +1816,7 @@
       <c r="G13" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="H13" s="20" t="s">
+      <c r="H13" s="17" t="s">
         <v>46</v>
       </c>
       <c r="I13" s="2" t="s">
@@ -1728,7 +1830,7 @@
       </c>
     </row>
     <row r="14" spans="1:16" ht="58.3" x14ac:dyDescent="0.4">
-      <c r="A14" s="17">
+      <c r="A14" s="14">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
@@ -1750,7 +1852,7 @@
       <c r="G14" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="H14" s="20" t="s">
+      <c r="H14" s="17" t="s">
         <v>46</v>
       </c>
       <c r="I14" s="2" t="s">
@@ -1762,7 +1864,7 @@
       <c r="K14" s="2"/>
     </row>
     <row r="15" spans="1:16" ht="58.3" x14ac:dyDescent="0.4">
-      <c r="A15" s="17">
+      <c r="A15" s="14">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
@@ -1784,7 +1886,7 @@
       <c r="G15" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="H15" s="20" t="s">
+      <c r="H15" s="17" t="s">
         <v>46</v>
       </c>
       <c r="I15" s="2" t="s">
@@ -1796,7 +1898,7 @@
       <c r="K15" s="2"/>
     </row>
     <row r="16" spans="1:16" ht="58.3" x14ac:dyDescent="0.4">
-      <c r="A16" s="17">
+      <c r="A16" s="14">
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
@@ -1818,7 +1920,7 @@
       <c r="G16" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="H16" s="20" t="s">
+      <c r="H16" s="17" t="s">
         <v>46</v>
       </c>
       <c r="I16" s="2" t="s">
@@ -1830,7 +1932,7 @@
       <c r="K16" s="2"/>
     </row>
     <row r="17" spans="1:11" ht="58.3" x14ac:dyDescent="0.4">
-      <c r="A17" s="17">
+      <c r="A17" s="14">
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
@@ -1852,7 +1954,7 @@
       <c r="G17" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="H17" s="20" t="s">
+      <c r="H17" s="17" t="s">
         <v>46</v>
       </c>
       <c r="I17" s="2" t="s">
@@ -1864,7 +1966,7 @@
       <c r="K17" s="2"/>
     </row>
     <row r="18" spans="1:11" ht="58.3" x14ac:dyDescent="0.4">
-      <c r="A18" s="17">
+      <c r="A18" s="14">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
@@ -1880,7 +1982,7 @@
       </c>
       <c r="F18" s="2"/>
       <c r="G18" s="2"/>
-      <c r="H18" s="20" t="s">
+      <c r="H18" s="17" t="s">
         <v>56</v>
       </c>
       <c r="I18" s="2" t="s">
@@ -1894,7 +1996,7 @@
       </c>
     </row>
     <row r="19" spans="1:11" ht="102" x14ac:dyDescent="0.4">
-      <c r="A19" s="17">
+      <c r="A19" s="14">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
@@ -1916,10 +2018,10 @@
       <c r="G19" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="H19" s="20" t="s">
-        <v>46</v>
-      </c>
-      <c r="I19" s="19" t="s">
+      <c r="H19" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="I19" s="16" t="s">
         <v>97</v>
       </c>
       <c r="J19" s="2" t="s">
@@ -1930,7 +2032,7 @@
       </c>
     </row>
     <row r="20" spans="1:11" ht="320.60000000000002" x14ac:dyDescent="0.4">
-      <c r="A20" s="17">
+      <c r="A20" s="14">
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
@@ -1952,7 +2054,7 @@
       <c r="G20" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="H20" s="20" t="s">
+      <c r="H20" s="17" t="s">
         <v>56</v>
       </c>
       <c r="I20" s="2" t="s">
@@ -1966,7 +2068,7 @@
       </c>
     </row>
     <row r="21" spans="1:11" ht="233.15" x14ac:dyDescent="0.4">
-      <c r="A21" s="17">
+      <c r="A21" s="14">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
@@ -1988,7 +2090,7 @@
       <c r="G21" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="H21" s="20" t="s">
+      <c r="H21" s="17" t="s">
         <v>56</v>
       </c>
       <c r="I21" s="2" t="s">
@@ -2002,7 +2104,7 @@
       </c>
     </row>
     <row r="22" spans="1:11" ht="43.75" x14ac:dyDescent="0.4">
-      <c r="A22" s="17">
+      <c r="A22" s="14">
         <f t="shared" si="0"/>
         <v>19</v>
       </c>
@@ -2024,7 +2126,7 @@
       <c r="G22" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="H22" s="20" t="s">
+      <c r="H22" s="17" t="s">
         <v>46</v>
       </c>
       <c r="I22" s="2" t="s">
@@ -2036,7 +2138,7 @@
       <c r="K22" s="2"/>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A23" s="17">
+      <c r="A23" s="14">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
@@ -2048,13 +2150,13 @@
       <c r="E23" s="2"/>
       <c r="F23" s="2"/>
       <c r="G23" s="2"/>
-      <c r="H23" s="20"/>
+      <c r="H23" s="17"/>
       <c r="I23" s="2"/>
       <c r="J23" s="2"/>
       <c r="K23" s="2"/>
     </row>
     <row r="24" spans="1:11" ht="58.3" x14ac:dyDescent="0.4">
-      <c r="A24" s="17">
+      <c r="A24" s="14">
         <f t="shared" si="0"/>
         <v>21</v>
       </c>
@@ -2076,7 +2178,7 @@
       <c r="G24" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="H24" s="20" t="s">
+      <c r="H24" s="17" t="s">
         <v>46</v>
       </c>
       <c r="I24" s="2" t="s">
@@ -2088,7 +2190,7 @@
       <c r="K24" s="2"/>
     </row>
     <row r="25" spans="1:11" ht="102" x14ac:dyDescent="0.4">
-      <c r="A25" s="17">
+      <c r="A25" s="14">
         <f t="shared" si="0"/>
         <v>22</v>
       </c>
@@ -2110,7 +2212,7 @@
       <c r="G25" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="H25" s="20" t="s">
+      <c r="H25" s="17" t="s">
         <v>46</v>
       </c>
       <c r="I25" s="2" t="s">
@@ -2122,7 +2224,7 @@
       <c r="K25" s="2"/>
     </row>
     <row r="26" spans="1:11" ht="102" x14ac:dyDescent="0.4">
-      <c r="A26" s="17">
+      <c r="A26" s="14">
         <f t="shared" si="0"/>
         <v>23</v>
       </c>
@@ -2144,7 +2246,7 @@
       <c r="G26" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="H26" s="20" t="s">
+      <c r="H26" s="17" t="s">
         <v>46</v>
       </c>
       <c r="I26" s="2" t="s">
@@ -2156,7 +2258,7 @@
       <c r="K26" s="2"/>
     </row>
     <row r="27" spans="1:11" ht="160.30000000000001" x14ac:dyDescent="0.4">
-      <c r="A27" s="17">
+      <c r="A27" s="14">
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
@@ -2178,7 +2280,7 @@
       <c r="G27" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="H27" s="20" t="s">
+      <c r="H27" s="17" t="s">
         <v>46</v>
       </c>
       <c r="I27" s="2" t="s">
@@ -2190,7 +2292,7 @@
       <c r="K27" s="2"/>
     </row>
     <row r="28" spans="1:11" ht="131.15" x14ac:dyDescent="0.4">
-      <c r="A28" s="17">
+      <c r="A28" s="14">
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
@@ -2212,7 +2314,7 @@
       <c r="G28" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="H28" s="20" t="s">
+      <c r="H28" s="17" t="s">
         <v>46</v>
       </c>
       <c r="I28" s="2" t="s">
@@ -2224,7 +2326,7 @@
       <c r="K28" s="2"/>
     </row>
     <row r="29" spans="1:11" ht="189.45" x14ac:dyDescent="0.4">
-      <c r="A29" s="17">
+      <c r="A29" s="14">
         <f t="shared" si="0"/>
         <v>26</v>
       </c>
@@ -2246,7 +2348,7 @@
       <c r="G29" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="H29" s="20" t="s">
+      <c r="H29" s="17" t="s">
         <v>46</v>
       </c>
       <c r="I29" s="2" t="s">
@@ -2258,7 +2360,7 @@
       <c r="K29" s="2"/>
     </row>
     <row r="30" spans="1:11" ht="218.6" x14ac:dyDescent="0.4">
-      <c r="A30" s="17">
+      <c r="A30" s="14">
         <f t="shared" si="0"/>
         <v>27</v>
       </c>
@@ -2280,7 +2382,7 @@
       <c r="G30" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="H30" s="20" t="s">
+      <c r="H30" s="17" t="s">
         <v>46</v>
       </c>
       <c r="I30" s="2" t="s">
@@ -2292,7 +2394,7 @@
       <c r="K30" s="2"/>
     </row>
     <row r="31" spans="1:11" ht="72.900000000000006" x14ac:dyDescent="0.4">
-      <c r="A31" s="17">
+      <c r="A31" s="14">
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
@@ -2312,7 +2414,7 @@
       <c r="G31" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="H31" s="20" t="s">
+      <c r="H31" s="17" t="s">
         <v>46</v>
       </c>
       <c r="I31" s="2" t="s">
@@ -2324,7 +2426,7 @@
       <c r="K31" s="2"/>
     </row>
     <row r="32" spans="1:11" ht="43.75" x14ac:dyDescent="0.4">
-      <c r="A32" s="17">
+      <c r="A32" s="14">
         <f t="shared" si="0"/>
         <v>29</v>
       </c>
@@ -2344,7 +2446,7 @@
       <c r="G32" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="H32" s="20" t="s">
+      <c r="H32" s="17" t="s">
         <v>46</v>
       </c>
       <c r="I32" s="2" t="s">
@@ -2356,7 +2458,7 @@
       <c r="K32" s="2"/>
     </row>
     <row r="33" spans="1:11" ht="145.75" x14ac:dyDescent="0.4">
-      <c r="A33" s="17">
+      <c r="A33" s="14">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
@@ -2376,7 +2478,7 @@
       <c r="G33" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="H33" s="20" t="s">
+      <c r="H33" s="17" t="s">
         <v>46</v>
       </c>
       <c r="I33" s="2" t="s">
@@ -2390,7 +2492,7 @@
       </c>
     </row>
     <row r="34" spans="1:11" ht="43.75" x14ac:dyDescent="0.4">
-      <c r="A34" s="17">
+      <c r="A34" s="14">
         <f t="shared" si="0"/>
         <v>31</v>
       </c>
@@ -2410,7 +2512,7 @@
       <c r="G34" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="H34" s="20" t="s">
+      <c r="H34" s="17" t="s">
         <v>46</v>
       </c>
       <c r="I34" s="2" t="s">
@@ -2422,7 +2524,7 @@
       <c r="K34" s="2"/>
     </row>
     <row r="35" spans="1:11" ht="43.75" x14ac:dyDescent="0.4">
-      <c r="A35" s="17">
+      <c r="A35" s="14">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
@@ -2442,7 +2544,7 @@
       <c r="G35" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="H35" s="20" t="s">
+      <c r="H35" s="17" t="s">
         <v>46</v>
       </c>
       <c r="I35" s="2" t="s">
@@ -2454,7 +2556,7 @@
       <c r="K35" s="2"/>
     </row>
     <row r="36" spans="1:11" ht="43.75" x14ac:dyDescent="0.4">
-      <c r="A36" s="17">
+      <c r="A36" s="14">
         <f t="shared" si="0"/>
         <v>33</v>
       </c>
@@ -2474,7 +2576,7 @@
       <c r="G36" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="H36" s="20" t="s">
+      <c r="H36" s="17" t="s">
         <v>46</v>
       </c>
       <c r="I36" s="2" t="s">
@@ -2486,7 +2588,7 @@
       <c r="K36" s="2"/>
     </row>
     <row r="37" spans="1:11" ht="145.75" x14ac:dyDescent="0.4">
-      <c r="A37" s="17">
+      <c r="A37" s="14">
         <f t="shared" si="0"/>
         <v>34</v>
       </c>
@@ -2506,7 +2608,7 @@
       <c r="G37" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="H37" s="20" t="s">
+      <c r="H37" s="17" t="s">
         <v>46</v>
       </c>
       <c r="I37" s="2" t="s">
@@ -2527,7 +2629,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{37BEB3A2-3F3B-40E8-964B-9CDD8DCD248B}">
-  <dimension ref="A1:P29"/>
+  <dimension ref="A1:P18"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="14.3828125" customWidth="1"/>
@@ -2543,42 +2645,42 @@
     <col min="11" max="11" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="9" t="s">
+    <row r="1" spans="1:16" s="21" customFormat="1" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="D1" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="E1" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="F1" s="10" t="s">
+      <c r="F1" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="G1" s="10" t="s">
+      <c r="G1" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="H1" s="10" t="s">
+      <c r="H1" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="I1" s="10" t="s">
+      <c r="I1" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="J1" s="10" t="s">
+      <c r="J1" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="K1" s="11" t="s">
+      <c r="K1" s="20" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:16" s="1" customFormat="1" ht="87.45" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:16" s="1" customFormat="1" ht="87.45" hidden="1" x14ac:dyDescent="0.4">
       <c r="A2" s="6"/>
       <c r="B2" s="7" t="s">
         <v>2</v>
@@ -2611,46 +2713,62 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:16" s="1" customFormat="1" ht="73.3" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A3" s="12"/>
-      <c r="B3" s="13" t="s">
+    <row r="3" spans="1:16" s="1" customFormat="1" ht="73.3" hidden="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A3" s="9"/>
+      <c r="B3" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="13" t="s">
+      <c r="C3" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="D3" s="13"/>
-      <c r="E3" s="13" t="s">
+      <c r="D3" s="10"/>
+      <c r="E3" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="F3" s="13" t="s">
+      <c r="F3" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="G3" s="13" t="s">
+      <c r="G3" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="H3" s="13"/>
-      <c r="I3" s="13"/>
-      <c r="J3" s="13" t="s">
+      <c r="H3" s="10"/>
+      <c r="I3" s="10"/>
+      <c r="J3" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="K3" s="14"/>
-    </row>
-    <row r="4" spans="1:16" ht="15" thickTop="1" x14ac:dyDescent="0.4">
+      <c r="K3" s="11"/>
+    </row>
+    <row r="4" spans="1:16" ht="204" x14ac:dyDescent="0.4">
       <c r="A4" s="5">
         <v>1</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>167</v>
       </c>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4"/>
-      <c r="I4" s="4"/>
-      <c r="J4" s="1"/>
+      <c r="C4" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>202</v>
+      </c>
+      <c r="H4" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>43</v>
+      </c>
       <c r="K4" s="1"/>
       <c r="L4" s="1"/>
       <c r="M4" s="1"/>
@@ -2658,144 +2776,256 @@
       <c r="O4" s="1"/>
       <c r="P4" s="1"/>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.4">
-      <c r="A5" s="17">
+    <row r="5" spans="1:16" ht="131.15" x14ac:dyDescent="0.4">
+      <c r="A5" s="14">
         <f>A4+1</f>
         <v>2</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
-      <c r="H5" s="20"/>
-      <c r="I5" s="2"/>
-      <c r="J5" s="2"/>
-      <c r="K5" s="18"/>
-      <c r="L5" s="1"/>
-      <c r="M5" s="1"/>
-      <c r="N5" s="1"/>
-      <c r="O5" s="1"/>
-      <c r="P5" s="1"/>
-    </row>
-    <row r="6" spans="1:16" ht="29.15" x14ac:dyDescent="0.4">
-      <c r="A6" s="17">
-        <f t="shared" ref="A6:A23" si="0">A5+1</f>
+      <c r="C5" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="H5" s="17" t="s">
+        <v>56</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="K5" s="2" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" ht="189.45" x14ac:dyDescent="0.4">
+      <c r="A6" s="14">
+        <f t="shared" ref="A6:A15" si="0">A5+1</f>
         <v>3</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>169</v>
       </c>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
-      <c r="H6" s="20"/>
-      <c r="I6" s="2"/>
-      <c r="J6" s="2"/>
-      <c r="K6" s="2"/>
-      <c r="L6" s="1"/>
-      <c r="M6" s="1"/>
-      <c r="N6" s="1"/>
-      <c r="O6" s="1"/>
-      <c r="P6" s="1"/>
-    </row>
-    <row r="7" spans="1:16" ht="42.9" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="17">
+      <c r="C6" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="H6" s="17" t="s">
+        <v>56</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" ht="233.15" x14ac:dyDescent="0.4">
+      <c r="A7" s="14">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
-      <c r="H7" s="20"/>
-      <c r="I7" s="2"/>
-      <c r="J7" s="2"/>
+      <c r="C7" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="H7" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>43</v>
+      </c>
       <c r="K7" s="2"/>
     </row>
-    <row r="8" spans="1:16" ht="181.3" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A8" s="17">
+    <row r="8" spans="1:16" ht="233.15" x14ac:dyDescent="0.4">
+      <c r="A8" s="14">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
-      <c r="H8" s="20"/>
-      <c r="I8" s="2"/>
-      <c r="J8" s="2"/>
+      <c r="C8" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="H8" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>43</v>
+      </c>
       <c r="K8" s="2"/>
     </row>
-    <row r="9" spans="1:16" ht="63.45" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A9" s="17">
+    <row r="9" spans="1:16" ht="87.45" x14ac:dyDescent="0.4">
+      <c r="A9" s="14">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
-      <c r="H9" s="20"/>
-      <c r="I9" s="2"/>
-      <c r="J9" s="2"/>
-      <c r="K9" s="2"/>
-    </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.4">
-      <c r="A10" s="17">
+      <c r="C9" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="H9" s="17" t="s">
+        <v>56</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="J9" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="K9" s="2" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" ht="87.45" x14ac:dyDescent="0.4">
+      <c r="A10" s="14">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>173</v>
       </c>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
-      <c r="G10" s="2"/>
-      <c r="H10" s="20"/>
-      <c r="I10" s="2"/>
-      <c r="J10" s="2"/>
-      <c r="K10" s="2"/>
-    </row>
-    <row r="11" spans="1:16" ht="29.15" x14ac:dyDescent="0.4">
-      <c r="A11" s="17">
+      <c r="C10" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="H10" s="17" t="s">
+        <v>56</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="J10" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="K10" s="2" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" ht="131.15" x14ac:dyDescent="0.4">
+      <c r="A11" s="14">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
-      <c r="G11" s="2"/>
-      <c r="H11" s="20"/>
-      <c r="I11" s="2"/>
-      <c r="J11" s="2"/>
-      <c r="K11" s="2"/>
+      <c r="C11" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="H11" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="J11" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="K11" s="2" t="s">
+        <v>45</v>
+      </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.4">
-      <c r="A12" s="17">
+      <c r="A12" s="14">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
@@ -2807,13 +3037,13 @@
       <c r="E12" s="2"/>
       <c r="F12" s="2"/>
       <c r="G12" s="2"/>
-      <c r="H12" s="20"/>
+      <c r="H12" s="17"/>
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
       <c r="K12" s="2"/>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.4">
-      <c r="A13" s="17">
+      <c r="A13" s="14">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
@@ -2825,18 +3055,13 @@
       <c r="E13" s="2"/>
       <c r="F13" s="2"/>
       <c r="G13" s="2"/>
-      <c r="H13" s="20"/>
+      <c r="H13" s="17"/>
       <c r="I13" s="2"/>
       <c r="J13" s="2"/>
-      <c r="K13" s="18"/>
-      <c r="L13" s="1"/>
-      <c r="M13" s="1"/>
-      <c r="N13" s="1"/>
-      <c r="O13" s="1"/>
-      <c r="P13" s="1"/>
+      <c r="K13" s="2"/>
     </row>
     <row r="14" spans="1:16" ht="29.15" x14ac:dyDescent="0.4">
-      <c r="A14" s="17">
+      <c r="A14" s="14">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
@@ -2848,18 +3073,13 @@
       <c r="E14" s="2"/>
       <c r="F14" s="2"/>
       <c r="G14" s="2"/>
-      <c r="H14" s="20"/>
+      <c r="H14" s="17"/>
       <c r="I14" s="2"/>
       <c r="J14" s="2"/>
       <c r="K14" s="2"/>
-      <c r="L14" s="1"/>
-      <c r="M14" s="1"/>
-      <c r="N14" s="1"/>
-      <c r="O14" s="1"/>
-      <c r="P14" s="1"/>
-    </row>
-    <row r="15" spans="1:16" ht="42.9" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A15" s="17">
+    </row>
+    <row r="15" spans="1:16" ht="29.15" x14ac:dyDescent="0.4">
+      <c r="A15" s="14">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
@@ -2871,186 +3091,19 @@
       <c r="E15" s="2"/>
       <c r="F15" s="2"/>
       <c r="G15" s="2"/>
-      <c r="H15" s="20"/>
+      <c r="H15" s="17"/>
       <c r="I15" s="2"/>
       <c r="J15" s="2"/>
       <c r="K15" s="2"/>
     </row>
-    <row r="16" spans="1:16" ht="181.3" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A16" s="17">
-        <f t="shared" si="0"/>
-        <v>13</v>
-      </c>
-      <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
-      <c r="G16" s="2"/>
-      <c r="H16" s="20"/>
-      <c r="I16" s="2"/>
-      <c r="J16" s="2"/>
-      <c r="K16" s="2"/>
-    </row>
-    <row r="17" spans="1:16" ht="63.45" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A17" s="17">
-        <f t="shared" si="0"/>
-        <v>14</v>
-      </c>
-      <c r="B17" s="2"/>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
-      <c r="F17" s="2"/>
-      <c r="G17" s="2"/>
-      <c r="H17" s="20"/>
-      <c r="I17" s="2"/>
-      <c r="J17" s="2"/>
-      <c r="K17" s="2"/>
-    </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.4">
-      <c r="A18" s="17">
-        <f t="shared" si="0"/>
-        <v>15</v>
-      </c>
-      <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
-      <c r="F18" s="2"/>
-      <c r="G18" s="2"/>
-      <c r="H18" s="20"/>
-      <c r="I18" s="2"/>
-      <c r="J18" s="2"/>
-      <c r="K18" s="2"/>
-    </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.4">
-      <c r="A19" s="17">
-        <f t="shared" si="0"/>
-        <v>16</v>
-      </c>
-      <c r="B19" s="2"/>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
-      <c r="E19" s="2"/>
-      <c r="F19" s="2"/>
-      <c r="G19" s="2"/>
-      <c r="H19" s="20"/>
-      <c r="I19" s="2"/>
-      <c r="J19" s="2"/>
-      <c r="K19" s="2"/>
-    </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.4">
-      <c r="A20" s="17">
-        <f t="shared" si="0"/>
-        <v>17</v>
-      </c>
-      <c r="B20" s="2"/>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
-      <c r="E20" s="2"/>
-      <c r="F20" s="2"/>
-      <c r="G20" s="2"/>
-      <c r="H20" s="20"/>
-      <c r="I20" s="2"/>
-      <c r="J20" s="2"/>
-      <c r="K20" s="2"/>
-    </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.4">
-      <c r="A21" s="17">
-        <f t="shared" si="0"/>
-        <v>18</v>
-      </c>
-      <c r="B21" s="2"/>
-      <c r="C21" s="2"/>
-      <c r="D21" s="2"/>
-      <c r="E21" s="2"/>
-      <c r="F21" s="2"/>
-      <c r="G21" s="2"/>
-      <c r="H21" s="20"/>
-      <c r="I21" s="2"/>
-      <c r="J21" s="2"/>
-      <c r="K21" s="18"/>
-      <c r="L21" s="1"/>
-      <c r="M21" s="1"/>
-      <c r="N21" s="1"/>
-      <c r="O21" s="1"/>
-      <c r="P21" s="1"/>
-    </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.4">
-      <c r="A22" s="17">
-        <f t="shared" si="0"/>
-        <v>19</v>
-      </c>
-      <c r="B22" s="2"/>
-      <c r="C22" s="2"/>
-      <c r="D22" s="2"/>
-      <c r="E22" s="2"/>
-      <c r="F22" s="2"/>
-      <c r="G22" s="2"/>
-      <c r="H22" s="20"/>
-      <c r="I22" s="2"/>
-      <c r="J22" s="2"/>
-      <c r="K22" s="2"/>
-      <c r="L22" s="1"/>
-      <c r="M22" s="1"/>
-      <c r="N22" s="1"/>
-      <c r="O22" s="1"/>
-      <c r="P22" s="1"/>
-    </row>
-    <row r="23" spans="1:16" ht="42.9" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A23" s="17">
-        <f t="shared" si="0"/>
-        <v>20</v>
-      </c>
-      <c r="B23" s="2"/>
-      <c r="C23" s="2"/>
-      <c r="D23" s="2"/>
-      <c r="E23" s="2"/>
-      <c r="F23" s="2"/>
-      <c r="G23" s="2"/>
-      <c r="H23" s="20"/>
-      <c r="I23" s="2"/>
-      <c r="J23" s="2"/>
-      <c r="K23" s="2"/>
-    </row>
-    <row r="24" spans="1:16" ht="181.3" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A24" s="17"/>
-      <c r="B24" s="2"/>
-      <c r="C24" s="2"/>
-      <c r="D24" s="2"/>
-      <c r="E24" s="2"/>
-      <c r="F24" s="2"/>
-      <c r="G24" s="2"/>
-      <c r="H24" s="20"/>
-      <c r="I24" s="2"/>
-      <c r="J24" s="2"/>
-      <c r="K24" s="2"/>
-    </row>
-    <row r="25" spans="1:16" ht="63.45" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A25" s="17"/>
-      <c r="B25" s="2"/>
-      <c r="C25" s="2"/>
-      <c r="D25" s="2"/>
-      <c r="E25" s="2"/>
-      <c r="F25" s="2"/>
-      <c r="G25" s="2"/>
-      <c r="H25" s="20"/>
-      <c r="I25" s="2"/>
-      <c r="J25" s="2"/>
-      <c r="K25" s="2"/>
-    </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.4">
-      <c r="A26" s="5"/>
-    </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.4">
-      <c r="A27" s="5"/>
-    </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.4">
-      <c r="A28" s="5"/>
-    </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.4">
-      <c r="A29" s="5"/>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.4">
+      <c r="A16" s="5"/>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A17" s="5"/>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A18" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3076,38 +3129,38 @@
     <col min="11" max="11" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="9" t="s">
+    <row r="1" spans="1:16" s="21" customFormat="1" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="D1" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="E1" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="F1" s="10" t="s">
+      <c r="F1" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="G1" s="10" t="s">
+      <c r="G1" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="H1" s="10" t="s">
+      <c r="H1" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="I1" s="10" t="s">
+      <c r="I1" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="J1" s="10" t="s">
+      <c r="J1" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="K1" s="11" t="s">
+      <c r="K1" s="20" t="s">
         <v>24</v>
       </c>
     </row>
@@ -3145,32 +3198,32 @@
       </c>
     </row>
     <row r="3" spans="1:16" s="1" customFormat="1" ht="73.3" hidden="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A3" s="12"/>
-      <c r="B3" s="13" t="s">
+      <c r="A3" s="9"/>
+      <c r="B3" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="13" t="s">
+      <c r="C3" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="D3" s="13"/>
-      <c r="E3" s="13" t="s">
+      <c r="D3" s="10"/>
+      <c r="E3" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="F3" s="13" t="s">
+      <c r="F3" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="G3" s="13" t="s">
+      <c r="G3" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="H3" s="13"/>
-      <c r="I3" s="13"/>
-      <c r="J3" s="13" t="s">
+      <c r="H3" s="10"/>
+      <c r="I3" s="10"/>
+      <c r="J3" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="K3" s="14"/>
+      <c r="K3" s="11"/>
     </row>
     <row r="4" spans="1:16" ht="204" x14ac:dyDescent="0.4">
-      <c r="A4" s="17">
+      <c r="A4" s="14">
         <v>1</v>
       </c>
       <c r="B4" s="2" t="s">
@@ -3191,7 +3244,7 @@
       <c r="G4" s="2" t="s">
         <v>181</v>
       </c>
-      <c r="H4" s="20" t="s">
+      <c r="H4" s="17" t="s">
         <v>46</v>
       </c>
       <c r="I4" s="2" t="s">
@@ -3208,7 +3261,7 @@
       <c r="P4" s="1"/>
     </row>
     <row r="5" spans="1:16" ht="181.3" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="17">
+      <c r="A5" s="14">
         <f>A4+1</f>
         <v>2</v>
       </c>
@@ -3230,7 +3283,7 @@
       <c r="G5" s="2" t="s">
         <v>181</v>
       </c>
-      <c r="H5" s="20" t="s">
+      <c r="H5" s="17" t="s">
         <v>46</v>
       </c>
       <c r="I5" s="2" t="s">
@@ -3244,7 +3297,7 @@
       </c>
     </row>
     <row r="6" spans="1:16" ht="102" x14ac:dyDescent="0.4">
-      <c r="A6" s="17">
+      <c r="A6" s="14">
         <f t="shared" ref="A6:A9" si="0">A5+1</f>
         <v>3</v>
       </c>
@@ -3266,7 +3319,7 @@
       <c r="G6" s="2" t="s">
         <v>187</v>
       </c>
-      <c r="H6" s="20" t="s">
+      <c r="H6" s="17" t="s">
         <v>46</v>
       </c>
       <c r="I6" s="2" t="s">
@@ -3278,7 +3331,7 @@
       <c r="K6" s="2"/>
     </row>
     <row r="7" spans="1:16" ht="116.6" x14ac:dyDescent="0.4">
-      <c r="A7" s="17">
+      <c r="A7" s="14">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
@@ -3300,7 +3353,7 @@
       <c r="G7" s="2" t="s">
         <v>189</v>
       </c>
-      <c r="H7" s="20" t="s">
+      <c r="H7" s="17" t="s">
         <v>46</v>
       </c>
       <c r="I7" s="2" t="s">
@@ -3314,7 +3367,7 @@
       </c>
     </row>
     <row r="8" spans="1:16" ht="174.9" x14ac:dyDescent="0.4">
-      <c r="A8" s="17">
+      <c r="A8" s="14">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
@@ -3336,7 +3389,7 @@
       <c r="G8" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="H8" s="20" t="s">
+      <c r="H8" s="17" t="s">
         <v>46</v>
       </c>
       <c r="I8" s="2" t="s">
@@ -3348,7 +3401,7 @@
       <c r="K8" s="2"/>
     </row>
     <row r="9" spans="1:16" ht="102" x14ac:dyDescent="0.4">
-      <c r="A9" s="17">
+      <c r="A9" s="14">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
@@ -3370,7 +3423,7 @@
       <c r="G9" s="2" t="s">
         <v>199</v>
       </c>
-      <c r="H9" s="20" t="s">
+      <c r="H9" s="17" t="s">
         <v>46</v>
       </c>
       <c r="I9" s="2" t="s">

</xml_diff>